<commit_message>
Upraven lean canvas dle nové monezitace a přidány slidy do prezentace
</commit_message>
<xml_diff>
--- a/Docs/naklady.xlsx
+++ b/Docs/naklady.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jumbo\team-7\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B8AB20-4342-475E-91D4-62B7FFED75C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2AD790-CC51-4E59-BA99-8916638615E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{19D1A740-1C33-4B9C-A256-A707425EC74D}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{19D1A740-1C33-4B9C-A256-A707425EC74D}"/>
   </bookViews>
   <sheets>
     <sheet name="Náklady na provoz" sheetId="1" r:id="rId1"/>

</xml_diff>